<commit_message>
Tillad formationsskift fra runde til runde for guld- og sølvhold
Guldhold genoptimerer nu fuldt ud hver runde over alle 7 formationer
(budget = kontanter + nuværende trups værdi), i stedet for at låse
formationen fra runde 1. Sølvholdets skift-søgning tillader nu også
tværposition-skift, valideret mod de tilladte formationer. Fælles
logik flyttet til holdet_lib.js (runGoldTrajectory/runSilverTrajectory)
og genbruges af ideal_guldhold.js, ideal_solvhold.js og ven_anbefalinger.js.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ideelle_hold_runde2.xlsx
+++ b/ideelle_hold_runde2.xlsx
@@ -493,16 +493,16 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Forsvar</v>
+        <v>Midtbane</v>
       </c>
       <c r="B6" t="str">
-        <v>Marcus Holmgren Pedersen</v>
+        <v>Ismaila Sarr</v>
       </c>
       <c r="C6" t="str">
-        <v>Norge</v>
+        <v>Senegal</v>
       </c>
       <c r="D6">
-        <v>221000</v>
+        <v>305000</v>
       </c>
       <c r="E6" t="str">
         <v/>
@@ -513,13 +513,13 @@
         <v>Midtbane</v>
       </c>
       <c r="B7" t="str">
-        <v>Ismaila Sarr</v>
+        <v>Nathan Saliba</v>
       </c>
       <c r="C7" t="str">
-        <v>Senegal</v>
+        <v>Canada</v>
       </c>
       <c r="D7">
-        <v>305000</v>
+        <v>272000</v>
       </c>
       <c r="E7" t="str">
         <v/>
@@ -530,13 +530,13 @@
         <v>Midtbane</v>
       </c>
       <c r="B8" t="str">
-        <v>Nathan Saliba</v>
+        <v>Luis Romo</v>
       </c>
       <c r="C8" t="str">
-        <v>Canada</v>
+        <v>Mexico</v>
       </c>
       <c r="D8">
-        <v>272000</v>
+        <v>265000</v>
       </c>
       <c r="E8" t="str">
         <v/>
@@ -547,13 +547,13 @@
         <v>Midtbane</v>
       </c>
       <c r="B9" t="str">
-        <v>Luis Romo</v>
+        <v>Mostafa Ziko</v>
       </c>
       <c r="C9" t="str">
-        <v>Mexico</v>
+        <v>Egypten</v>
       </c>
       <c r="D9">
-        <v>265000</v>
+        <v>254000</v>
       </c>
       <c r="E9" t="str">
         <v/>
@@ -1243,13 +1243,13 @@
         <v>Angreb</v>
       </c>
       <c r="B12" t="str">
-        <v>Mikel Oyarzabal</v>
+        <v>Ayase Ueda</v>
       </c>
       <c r="C12" t="str">
-        <v>Spanien</v>
+        <v>Japan</v>
       </c>
       <c r="D12">
-        <v>415000</v>
+        <v>425000</v>
       </c>
       <c r="E12" t="str">
         <v/>
@@ -1673,13 +1673,13 @@
         <v>Angreb</v>
       </c>
       <c r="B12" t="str">
-        <v>Ayase Ueda</v>
+        <v>Deniz Undav</v>
       </c>
       <c r="C12" t="str">
-        <v>Japan</v>
+        <v>Tyskland</v>
       </c>
       <c r="D12">
-        <v>425000</v>
+        <v>385000</v>
       </c>
       <c r="E12" t="str">
         <v/>
@@ -1735,13 +1735,13 @@
         <v>Forsvar</v>
       </c>
       <c r="B3" t="str">
-        <v>Willian Pacho</v>
+        <v>Daniel Muñoz</v>
       </c>
       <c r="C3" t="str">
-        <v>Ecuador</v>
+        <v>Colombia</v>
       </c>
       <c r="D3">
-        <v>72000</v>
+        <v>340000</v>
       </c>
       <c r="E3" t="str">
         <v/>
@@ -1752,13 +1752,13 @@
         <v>Forsvar</v>
       </c>
       <c r="B4" t="str">
-        <v>Caleb Yirenkyi</v>
+        <v>Willian Pacho</v>
       </c>
       <c r="C4" t="str">
-        <v>Ghana</v>
+        <v>Ecuador</v>
       </c>
       <c r="D4">
-        <v>62000</v>
+        <v>72000</v>
       </c>
       <c r="E4" t="str">
         <v/>
@@ -1769,13 +1769,13 @@
         <v>Forsvar</v>
       </c>
       <c r="B5" t="str">
-        <v>Jonathan Tah</v>
+        <v>Caleb Yirenkyi</v>
       </c>
       <c r="C5" t="str">
-        <v>Tyskland</v>
+        <v>Ghana</v>
       </c>
       <c r="D5">
-        <v>44000</v>
+        <v>62000</v>
       </c>
       <c r="E5" t="str">
         <v/>
@@ -1783,16 +1783,16 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Midtbane</v>
+        <v>Forsvar</v>
       </c>
       <c r="B6" t="str">
-        <v>Florian Wirtz</v>
+        <v>Jonathan Tah</v>
       </c>
       <c r="C6" t="str">
         <v>Tyskland</v>
       </c>
       <c r="D6">
-        <v>54000</v>
+        <v>44000</v>
       </c>
       <c r="E6" t="str">
         <v/>
@@ -1803,13 +1803,13 @@
         <v>Midtbane</v>
       </c>
       <c r="B7" t="str">
-        <v>Jamal Musiala</v>
+        <v>Florian Wirtz</v>
       </c>
       <c r="C7" t="str">
         <v>Tyskland</v>
       </c>
       <c r="D7">
-        <v>24000</v>
+        <v>54000</v>
       </c>
       <c r="E7" t="str">
         <v/>
@@ -1871,13 +1871,13 @@
         <v>Angreb</v>
       </c>
       <c r="B11" t="str">
-        <v>Cody Gakpo</v>
+        <v>Brian Brobbey</v>
       </c>
       <c r="C11" t="str">
         <v>Holland</v>
       </c>
       <c r="D11">
-        <v>437000</v>
+        <v>354000</v>
       </c>
       <c r="E11" t="str">
         <v/>
@@ -1888,13 +1888,13 @@
         <v>Angreb</v>
       </c>
       <c r="B12" t="str">
-        <v>Ayase Ueda</v>
+        <v>Enner Valencia</v>
       </c>
       <c r="C12" t="str">
-        <v>Japan</v>
+        <v>Ecuador</v>
       </c>
       <c r="D12">
-        <v>425000</v>
+        <v>62000</v>
       </c>
       <c r="E12" t="str">
         <v/>
@@ -1950,13 +1950,13 @@
         <v>Forsvar</v>
       </c>
       <c r="B3" t="str">
-        <v>Daniel Muñoz</v>
+        <v>Pau Cubarsi</v>
       </c>
       <c r="C3" t="str">
-        <v>Colombia</v>
+        <v>Spanien</v>
       </c>
       <c r="D3">
-        <v>340000</v>
+        <v>122000</v>
       </c>
       <c r="E3" t="str">
         <v/>
@@ -1967,13 +1967,13 @@
         <v>Forsvar</v>
       </c>
       <c r="B4" t="str">
-        <v>Pau Cubarsi</v>
+        <v>Jules Kounde</v>
       </c>
       <c r="C4" t="str">
-        <v>Spanien</v>
+        <v>Frankrig</v>
       </c>
       <c r="D4">
-        <v>122000</v>
+        <v>112000</v>
       </c>
       <c r="E4" t="str">
         <v/>
@@ -1984,13 +1984,13 @@
         <v>Forsvar</v>
       </c>
       <c r="B5" t="str">
-        <v>Jules Kounde</v>
+        <v>Cesar Montes</v>
       </c>
       <c r="C5" t="str">
-        <v>Frankrig</v>
+        <v>Mexico</v>
       </c>
       <c r="D5">
-        <v>112000</v>
+        <v>-5000</v>
       </c>
       <c r="E5" t="str">
         <v/>
@@ -2001,13 +2001,13 @@
         <v>Midtbane</v>
       </c>
       <c r="B6" t="str">
-        <v>Mahmoud Trezeguet</v>
+        <v>Ismaila Sarr</v>
       </c>
       <c r="C6" t="str">
-        <v>Egypten</v>
+        <v>Senegal</v>
       </c>
       <c r="D6">
-        <v>192000</v>
+        <v>305000</v>
       </c>
       <c r="E6" t="str">
         <v/>
@@ -2018,13 +2018,13 @@
         <v>Midtbane</v>
       </c>
       <c r="B7" t="str">
-        <v>Alexis Mac Allister</v>
+        <v>Mahmoud Trezeguet</v>
       </c>
       <c r="C7" t="str">
-        <v>Argentina</v>
+        <v>Egypten</v>
       </c>
       <c r="D7">
-        <v>52000</v>
+        <v>192000</v>
       </c>
       <c r="E7" t="str">
         <v/>
@@ -2035,13 +2035,13 @@
         <v>Midtbane</v>
       </c>
       <c r="B8" t="str">
-        <v>Jamal Musiala</v>
+        <v>Alexis Mac Allister</v>
       </c>
       <c r="C8" t="str">
-        <v>Tyskland</v>
+        <v>Argentina</v>
       </c>
       <c r="D8">
-        <v>24000</v>
+        <v>52000</v>
       </c>
       <c r="E8" t="str">
         <v/>
@@ -2052,13 +2052,13 @@
         <v>Midtbane</v>
       </c>
       <c r="B9" t="str">
-        <v>Alvaro Fidalgo</v>
+        <v>Jamal Musiala</v>
       </c>
       <c r="C9" t="str">
-        <v>Mexico</v>
+        <v>Tyskland</v>
       </c>
       <c r="D9">
-        <v>-5000</v>
+        <v>24000</v>
       </c>
       <c r="E9" t="str">
         <v/>

</xml_diff>

<commit_message>
Fix: vennes faktiske runde-trup blev fejlagtigt om-optimeret i guldhold-anbefalinger
runGoldTrajectory genoptimerede selve fromRound, selv når en kendt faktisk
trup (en vens reelle hold) var givet som baseSquad. Det betød at allerede
ejede spillere med lav vækst i den runde (fx Oyarzabal i runde 1) kunne
blive "skiftet ud" i en hypotetisk om-optimering af en allerede afsluttet
runde, før den efterfølgende runde overhovedet blev beregnet — så de
mistede deres gebyrfri status i den faktiske anbefaling. Nu behandles en
given baseSquad som et fast historisk udgangspunkt, og om-optimering
starter først fra runden efter.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ideelle_hold_runde2.xlsx
+++ b/ideelle_hold_runde2.xlsx
@@ -1243,13 +1243,13 @@
         <v>Angreb</v>
       </c>
       <c r="B12" t="str">
-        <v>Ayase Ueda</v>
+        <v>Mikel Oyarzabal</v>
       </c>
       <c r="C12" t="str">
-        <v>Japan</v>
+        <v>Spanien</v>
       </c>
       <c r="D12">
-        <v>425000</v>
+        <v>415000</v>
       </c>
       <c r="E12" t="str">
         <v/>

</xml_diff>